<commit_message>
test(excel): the held-out keep cases of the AutoFilter, as Excel did and opened them
The four answers are the ones predicted; the filter database, which Excel moves as a name,
differs where the AutoFilter stays and the name stretches.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/excel/keep/struct-open/filter-delete-header.xlsx
+++ b/test/excel/keep/struct-open/filter-delete-header.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fkeep-60271/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mike/Library/Containers/com.microsoft.Excel/Data/tmp/fkeep-68964/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C9A9876-DA5B-B74A-B059-CC878F184769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0D035C8-EDB9-884C-92BC-DF0799681929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,9 +17,6 @@
     <sheet name="Pivot" sheetId="2" r:id="rId2"/>
     <sheet name="Plain" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Data!$A$1:$C$20</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -680,7 +677,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C20" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>